<commit_message>
docs: remove add rms norm screenshot placeholders
</commit_message>
<xml_diff>
--- a/third_party/ascend/tutorials/add_rms_norm/AddRmsNorm算子自验证报告.xlsx
+++ b/third_party/ascend/tutorials/add_rms_norm/AddRmsNorm算子自验证报告.xlsx
@@ -555,12 +555,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -775,12 +775,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -830,12 +830,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -885,12 +885,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -940,12 +940,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -995,12 +995,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1160,12 +1160,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1215,12 +1215,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1325,12 +1325,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1380,12 +1380,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1435,12 +1435,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1545,12 +1545,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1600,12 +1600,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1655,12 +1655,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1820,12 +1820,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1875,12 +1875,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2040,12 +2040,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2095,12 +2095,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2205,12 +2205,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2315,12 +2315,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2370,12 +2370,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2425,12 +2425,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2480,12 +2480,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2535,12 +2535,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2590,12 +2590,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2700,12 +2700,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2755,12 +2755,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2810,12 +2810,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2865,12 +2865,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2920,12 +2920,12 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -2975,12 +2975,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -3030,12 +3030,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -3085,12 +3085,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -3140,12 +3140,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -3195,12 +3195,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3250,12 +3250,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3305,12 +3305,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3360,12 +3360,12 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3415,12 +3415,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3470,12 +3470,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -3525,12 +3525,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3580,12 +3580,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -3635,12 +3635,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -3690,12 +3690,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -3745,12 +3745,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3800,12 +3800,12 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -3855,12 +3855,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -3910,12 +3910,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -3965,12 +3965,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -4020,12 +4020,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -4075,12 +4075,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -4185,12 +4185,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -4240,12 +4240,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -4350,12 +4350,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -4405,12 +4405,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4460,12 +4460,12 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -4515,12 +4515,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -4570,12 +4570,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -4625,12 +4625,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -4735,12 +4735,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4790,12 +4790,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -4845,12 +4845,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -4900,12 +4900,12 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>见“日志证据”工作表及外部截图</t>
+          <t>见“日志证据”工作表</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">

</xml_diff>